<commit_message>
Update soccer trades 2026-07-31 01:03:48 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/LigaPro/trades.xlsx
+++ b/data/sxbet/ligas/LigaPro/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,102 +531,94 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>9.84</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.4363</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>250.01</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.4812</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Manta FC vs Mushuc Runa</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Mushuc Runa</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19605615</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785441463</t>
+          <t>1785459616</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>519.501299</t>
+          <t>22.555874</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,102 +635,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.435</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>141.16</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.3438</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Manta FC vs Mushuc Runa</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Mushuc Runa</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19605615</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785441440</t>
+          <t>1785459612</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>410.647273</t>
+          <t>45.977011</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,110 +739,1062 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.6173</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.4087</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1785459609</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>1.510214</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1785459608</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>112.676056</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1785459600</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>281.690141</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1785459599</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>45.070423</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>56.338028</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>22.535211</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>133.14</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.3475</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1785459478</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>383.136691</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>250.01</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.4812</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1785441463</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>519.501299</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>141.16</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1785441440</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>410.647273</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>0x6599044f3d4d50487489b07a035618092f1d03440ffd54856dcd903844650bb5</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>1.2575</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Tecnico U.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>L19606829</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>1785344362</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>1785619800</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>3.883495</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-01 19:02:56 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/LigaPro/trades.xlsx
+++ b/data/sxbet/ligas/LigaPro/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
+          <t>0xcac4d184a3b30b230068ae9c913c5c20aa85bbc70c10395795d8dd47887baf38</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,52 +546,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.24999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.5025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Universidad Catolica del Ecuador -1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785586109</t>
+          <t>1785608052</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.48137</t>
+          <t>19.900498</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
+          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>115.96999</t>
+          <t>1.24999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785581613</t>
+          <t>1785586109</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>233.692675</t>
+          <t>2.48137</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
+          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>115.97</t>
+          <t>115.96999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785579320</t>
+          <t>1785581613</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>233.692695</t>
+          <t>233.692675</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
+          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16.07</t>
+          <t>115.97</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -899,27 +907,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +952,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785559247</t>
+          <t>1785579320</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>29.554023</t>
+          <t>233.692695</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
+          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -992,7 +1000,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -1018,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1075,28 +1083,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
+          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>16.07</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LigaPro</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1107,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1152,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785559217</t>
+          <t>1785559247</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.909308</t>
+          <t>29.554023</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,28 +1187,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
+          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>15.99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1211,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1256,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785559203</t>
+          <t>1785559217</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>29.474654</t>
+          <t>1.909308</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
+          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1304,7 +1312,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1330,7 +1338,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1387,7 +1395,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
+          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1398,17 +1406,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.83</t>
+          <t>15.99</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1434,7 +1442,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1464,7 +1472,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785559136</t>
+          <t>1785559203</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1474,7 +1482,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>29.314815</t>
+          <t>29.474654</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,7 +1499,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
+          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1512,7 +1520,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1538,7 +1546,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1568,7 +1576,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785559135</t>
+          <t>1785559136</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1595,7 +1603,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
+          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1606,17 +1614,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>15.83</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1642,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1672,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785559114</t>
+          <t>1785559135</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1682,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.314815</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1699,7 +1707,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
+          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1720,7 +1728,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1746,7 +1754,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1803,7 +1811,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
+          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1880,7 +1888,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785559105</t>
+          <t>1785559114</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1907,7 +1915,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
+          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1928,7 +1936,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1954,7 +1962,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2011,18 +2019,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
+          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>173.57</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2088,7 +2096,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785557644</t>
+          <t>1785559105</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2098,7 +2106,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>322.92093</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2115,7 +2123,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
+          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2136,7 +2144,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2162,7 +2170,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2192,7 +2200,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785557643</t>
+          <t>1785557644</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2219,7 +2227,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
+          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2227,31 +2235,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.34</t>
+          <t>173.57</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4062</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785540081</t>
+          <t>1785557643</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>322.92093</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2331,12 +2331,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
+          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2346,22 +2346,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.34</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.4062</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2371,27 +2371,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2416,17 +2416,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785524760</t>
+          <t>1785540081</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>3.018868</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2443,15 +2443,19 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
+          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>1</t>
@@ -2459,7 +2463,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2467,7 +2471,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2475,27 +2483,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Emelec vs Aucas</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Emelec</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19607503</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2520,17 +2528,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785513340</t>
+          <t>1785524760</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1785628800</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.691332</t>
+          <t>3.018868</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2547,7 +2555,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
+          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2563,7 +2571,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.6825</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2579,27 +2587,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2624,17 +2632,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785513160</t>
+          <t>1785513340</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.465201</t>
+          <t>1.691332</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2651,28 +2659,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
+          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>18.41999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.6825</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>LigaPro</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2698,7 +2706,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2728,7 +2736,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785497374</t>
+          <t>1785513160</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2738,7 +2746,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>33.26409</t>
+          <t>1.465201</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2755,7 +2763,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
+          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2763,54 +2771,46 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>18.41999</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3738</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Libertad FC vs Orense Sporting Club</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>Orense Sporting Club</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Libertad FC</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Orense Sporting Club</t>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
+          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785497256</t>
+          <t>1785497374</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>4.120401</t>
+          <t>33.26409</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
+          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>15.65</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785497255</t>
+          <t>1785497256</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>41.87291</t>
+          <t>4.120401</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2979,7 +2979,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
+          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2994,29 +2994,29 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>15.65</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.3738</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Orense Sporting Club</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Libertad FC 0</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>Libertad FC vs Orense Sporting Club</t>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
+          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785487800</t>
+          <t>1785497255</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>7.543424</t>
+          <t>41.87291</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3091,31 +3091,39 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
+          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Libertad FC 0</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3123,27 +3131,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3168,17 +3176,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785460511</t>
+          <t>1785487800</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>7.543424</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3195,18 +3203,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
+          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3272,7 +3280,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785460290</t>
+          <t>1785460511</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3282,7 +3290,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>26.122449</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3299,28 +3307,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
+          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.44982</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3331,27 +3339,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3376,17 +3384,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785459886</t>
+          <t>1785460290</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>0.6426</t>
+          <t>26.122449</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3403,23 +3411,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
+          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>463.04</t>
+          <t>0.44982</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3480,7 +3488,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785459772</t>
+          <t>1785459886</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3490,7 +3498,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>712.369231</t>
+          <t>0.6426</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3507,28 +3515,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
+          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>9.84</t>
+          <t>463.04</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -3539,27 +3547,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3584,17 +3592,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785459616</t>
+          <t>1785459772</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>22.555874</t>
+          <t>712.369231</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3611,23 +3619,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
+          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9.84</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3688,7 +3696,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785459612</t>
+          <t>1785459616</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3698,7 +3706,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>45.977011</t>
+          <t>22.555874</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3715,23 +3723,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
+          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.6173</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3792,7 +3800,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785459609</t>
+          <t>1785459612</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3802,7 +3810,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.510214</t>
+          <t>45.977011</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3819,23 +3827,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
+          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0.6173</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3896,7 +3904,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785459608</t>
+          <t>1785459609</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3906,7 +3914,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>112.676056</t>
+          <t>1.510214</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3923,18 +3931,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
+          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4000,7 +4008,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785459600</t>
+          <t>1785459608</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4010,7 +4018,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>281.690141</t>
+          <t>112.676056</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4027,18 +4035,18 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
+          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4104,7 +4112,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785459599</t>
+          <t>1785459600</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4114,7 +4122,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>45.070423</t>
+          <t>281.690141</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4131,18 +4139,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4208,7 +4216,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785459589</t>
+          <t>1785459599</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4218,7 +4226,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>56.338028</t>
+          <t>45.070423</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4235,18 +4243,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4322,7 +4330,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>56.338028</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4339,23 +4347,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>133.14</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.3475</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4371,27 +4379,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4416,17 +4424,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785459478</t>
+          <t>1785459589</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>383.136691</t>
+          <t>22.535211</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4443,54 +4451,46 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>250.01</t>
+          <t>133.14</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.3475</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>Manta FC</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Manta FC vs Mushuc Runa</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Mushuc Runa</t>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785441463</t>
+          <t>1785459478</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>519.501299</t>
+          <t>383.136691</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4555,7 +4555,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4570,17 +4570,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>141.16</t>
+          <t>250.01</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4812</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785441440</t>
+          <t>1785441463</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>410.647273</t>
+          <t>519.501299</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4667,110 +4667,222 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>141.16</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1785441440</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>410.647273</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>0x6599044f3d4d50487489b07a035618092f1d03440ffd54856dcd903844650bb5</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>1.2575</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Tecnico U.</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>L19606829</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
         <is>
           <t>1785344362</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="S42" t="inlineStr">
         <is>
           <t>1785619800</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>3.883495</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-01 21:03:36 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/LigaPro/trades.xlsx
+++ b/data/sxbet/ligas/LigaPro/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xcac4d184a3b30b230068ae9c913c5c20aa85bbc70c10395795d8dd47887baf38</t>
+          <t>0x1c5449fdfedcee8971c0c384741afccf1819625941cea175c42c57045be09079</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5025</t>
+          <t>1.1525</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Universidad Catolica del Ecuador -1</t>
-        </is>
-      </c>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xc4044a0346c09a988a8646f1c19fcf4f0aebf02dd86358ff869417e13a149799</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785608052</t>
+          <t>1785617083</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>19.900498</t>
+          <t>11.344262</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
+          <t>0x49fe40db9721a6aaa44c12cdaa59de055cc21b9adc2a34ca866505256192b968</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,59 +643,51 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.24999</t>
+          <t>98</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.875</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785586109</t>
+          <t>1785616859</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2.48137</t>
+          <t>112.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
+          <t>0x4d5eee136de8446546eda81cbb34b3151a02e3a65539b580d186d7b15e7a047c</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,52 +754,52 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>115.96999</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.1287</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Tecnico U.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -840,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785581613</t>
+          <t>1785616850</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>233.692675</t>
+          <t>108.737864</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,67 +851,59 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
+          <t>0xd36df2627cc88fab7fdc1af73b8bcb3c0bf72929e79cf6bd4528a73bb336310c</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>115.97</t>
+          <t>38.02995</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.8588</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -952,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785579320</t>
+          <t>1785616283</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>233.692695</t>
+          <t>44.28524</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,31 +955,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
+          <t>0x5003aa71c29014639de94cd36c0d56636b10b1886f45c744d5d916eb60a6228c</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>16.07</t>
+          <t>8.00529</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1026,7 +1010,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1040,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785559247</t>
+          <t>1785615140</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1050,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>29.554023</t>
+          <t>34.24723</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,31 +1067,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
+          <t>0x47ab07234e0925e967962637a863ed524a79d48b9d461f04f5d7dcb51a9077bd</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16.07</t>
+          <t>8.01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1130,7 +1122,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1160,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785559247</t>
+          <t>1785615140</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>29.554023</t>
+          <t>34.451613</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,15 +1179,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
+          <t>0x4a0fce837f4b39328cc4cb76d4060e94a4597f4078a1ad0dff75a038c5d092c3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1203,43 +1199,47 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785559217</t>
+          <t>1785615126</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.909308</t>
+          <t>4.278075</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,28 +1291,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
+          <t>0xe7448cde3292b98680d8d685555b200090ccc908e6930965d17be8e6401d5629</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15.99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.8325</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1323,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xb4df2c601601b81281545002a7ee9a847a424801fa9f9ea09b68e930c647c2b2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785559203</t>
+          <t>1785613773</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>29.474654</t>
+          <t>1.201201</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,23 +1395,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
+          <t>0xcac4d184a3b30b230068ae9c913c5c20aa85bbc70c10395795d8dd47887baf38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15.99</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.5025</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1419,7 +1423,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Universidad Catolica del Ecuador -1</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1472,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785559203</t>
+          <t>1785608052</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1482,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>29.474654</t>
+          <t>19.900498</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,31 +1507,39 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
+          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>15.83</t>
+          <t>1.24999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1531,27 +1547,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1576,17 +1592,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785559136</t>
+          <t>1785586109</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>29.314815</t>
+          <t>2.48137</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,7 +1619,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
+          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1611,23 +1627,31 @@
           <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15.83</t>
+          <t>115.96999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1635,27 +1659,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1680,17 +1704,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785559135</t>
+          <t>1785581613</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>29.314815</t>
+          <t>233.692675</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,31 +1731,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
+          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>115.97</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1739,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1784,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785559114</t>
+          <t>1785579320</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>233.692695</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1811,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
+          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1822,17 +1854,17 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>16.07</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1858,7 +1890,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1888,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785559114</t>
+          <t>1785559247</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1898,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.554023</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1915,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
+          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1926,12 +1958,12 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>16.07</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1992,7 +2024,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785559105</t>
+          <t>1785559247</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2002,7 +2034,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.554023</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2019,28 +2051,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
+          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2051,27 +2083,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2096,17 +2128,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785559105</t>
+          <t>1785559217</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>1.909308</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2123,23 +2155,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
+          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>173.57</t>
+          <t>15.99</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2200,7 +2232,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785557644</t>
+          <t>1785559203</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2210,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>322.92093</t>
+          <t>29.474654</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2227,23 +2259,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
+          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>173.57</t>
+          <t>15.99</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2304,7 +2336,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785557643</t>
+          <t>1785559203</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2314,7 +2346,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>322.92093</t>
+          <t>29.474654</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2331,39 +2363,31 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
+          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.34</t>
+          <t>15.83</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4062</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2386,7 +2410,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2416,7 +2440,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785540081</t>
+          <t>1785559136</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2426,7 +2450,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>29.314815</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2443,39 +2467,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
+          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.83</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Libertad FC</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2483,27 +2499,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2528,17 +2544,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785524760</t>
+          <t>1785559135</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>3.018868</t>
+          <t>29.314815</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2555,28 +2571,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
+          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2587,27 +2603,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Emelec vs Aucas</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Emelec</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19607503</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2632,17 +2648,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785513340</t>
+          <t>1785559114</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1785628800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.691332</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2659,28 +2675,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
+          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.6825</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2691,27 +2707,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2736,17 +2752,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785513160</t>
+          <t>1785559114</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1.465201</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2763,28 +2779,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
+          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>18.41999</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>LigaPro</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -2795,27 +2811,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2840,17 +2856,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785497374</t>
+          <t>1785559105</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>33.26409</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2867,39 +2883,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
+          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3738</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Orense Sporting Club</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2907,27 +2915,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2952,17 +2960,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785497256</t>
+          <t>1785559105</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>4.120401</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2979,7 +2987,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
+          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2987,31 +2995,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>15.65</t>
+          <t>173.57</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.3738</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Orense Sporting Club</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3019,27 +3019,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3064,17 +3064,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785497255</t>
+          <t>1785557644</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>41.87291</t>
+          <t>322.92093</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3091,7 +3091,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
+          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3099,59 +3099,51 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>173.57</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Libertad FC 0</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3176,17 +3168,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785487800</t>
+          <t>1785557643</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>7.543424</t>
+          <t>322.92093</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3203,31 +3195,39 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
+          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.34</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.4062</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3235,27 +3235,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3280,17 +3280,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785460511</t>
+          <t>1785540081</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3307,31 +3307,39 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
+          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3339,27 +3347,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3384,17 +3392,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785460290</t>
+          <t>1785524760</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>26.122449</t>
+          <t>3.018868</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3411,23 +3419,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
+          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.44982</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3443,27 +3451,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3488,17 +3496,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785459886</t>
+          <t>1785513340</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>0.6426</t>
+          <t>1.691332</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3515,23 +3523,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
+          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>463.04</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.6825</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3547,27 +3555,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3592,17 +3600,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785459772</t>
+          <t>1785513160</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>712.369231</t>
+          <t>1.465201</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3619,28 +3627,28 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
+          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>9.84</t>
+          <t>18.41999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -3651,27 +3659,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3696,17 +3704,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785459616</t>
+          <t>1785497374</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>22.555874</t>
+          <t>33.26409</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3723,31 +3731,39 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
+          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.3738</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Orense Sporting Club</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3755,27 +3771,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3800,17 +3816,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785459612</t>
+          <t>1785497256</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>45.977011</t>
+          <t>4.120401</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3827,31 +3843,39 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
+          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.6173</t>
+          <t>15.65</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.3738</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Orense Sporting Club</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3859,27 +3883,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3904,17 +3928,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785459609</t>
+          <t>1785497255</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1.510214</t>
+          <t>41.87291</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3931,31 +3955,39 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
+          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Libertad FC 0</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3963,27 +3995,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4008,17 +4040,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785459608</t>
+          <t>1785487800</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>112.676056</t>
+          <t>7.543424</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4035,23 +4067,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
+          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4112,7 +4144,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785459600</t>
+          <t>1785460511</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4122,7 +4154,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>281.690141</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4139,23 +4171,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
+          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4216,7 +4248,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785459599</t>
+          <t>1785460290</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4226,7 +4258,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>45.070423</t>
+          <t>26.122449</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4243,28 +4275,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0.44982</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4275,27 +4307,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4320,17 +4352,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785459589</t>
+          <t>1785459886</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>56.338028</t>
+          <t>0.6426</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4347,28 +4379,28 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>463.04</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -4379,27 +4411,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4424,17 +4456,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785459589</t>
+          <t>1785459772</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>712.369231</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4451,23 +4483,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>133.14</t>
+          <t>9.84</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.3475</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4483,27 +4515,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4528,17 +4560,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785459478</t>
+          <t>1785459616</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>383.136691</t>
+          <t>22.555874</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4555,67 +4587,59 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>250.01</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4640,17 +4664,17 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785441463</t>
+          <t>1785459612</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>519.501299</t>
+          <t>45.977011</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4667,39 +4691,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>141.16</t>
+          <t>0.6173</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -4707,27 +4723,27 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4752,17 +4768,17 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785441440</t>
+          <t>1785459609</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>410.647273</t>
+          <t>1.510214</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4779,110 +4795,958 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1785459608</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>112.676056</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1785459600</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>281.690141</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1785459599</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>45.070423</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>56.338028</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>22.535211</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>133.14</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.3475</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1785459478</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>383.136691</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>250.01</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.4812</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1785441463</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>519.501299</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>141.16</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1785441440</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>410.647273</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>0x6599044f3d4d50487489b07a035618092f1d03440ffd54856dcd903844650bb5</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>1.2575</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Tecnico U.</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>L19606829</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
         <is>
           <t>1785344362</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>1785619800</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>3.883495</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-02 00:03:38 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/LigaPro/trades.xlsx
+++ b/data/sxbet/ligas/LigaPro/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V50"/>
+  <dimension ref="A1:V55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x1c5449fdfedcee8971c0c384741afccf1819625941cea175c42c57045be09079</t>
+          <t>0xe7e31dcf4e7091b0016161d9c81726ff15809ad88271acf1824432a40d628393</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>24.94998</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.1525</t>
+          <t>1.7375</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LigaPro</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xc4044a0346c09a988a8646f1c19fcf4f0aebf02dd86358ff869417e13a149799</t>
+          <t>0xbef81e804b45a008094d3ed28e67d3330de2ca8be595e69a04b9ef716d1b1ec9</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785617083</t>
+          <t>1785625675</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>11.344262</t>
+          <t>33.830481</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x49fe40db9721a6aaa44c12cdaa59de055cc21b9adc2a34ca866505256192b968</t>
+          <t>0x12b6130505cc8a8edf5b6b4633ba05d9b11cdfa9fac4d8bee6b88abd448c05b2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -646,12 +646,12 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>18.03999</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.875</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -667,27 +667,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
+          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +712,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785616859</t>
+          <t>1785623924</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>112.0</t>
+          <t>31.579851</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,12 +739,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x4d5eee136de8446546eda81cbb34b3151a02e3a65539b580d186d7b15e7a047c</t>
+          <t>0xcc3b3eaa312e1ba91ace2a7e33152f89d15f90298b8362a11344d1642edf31a5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1.01902</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1287</t>
+          <t>1.3088</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -779,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
+          <t>0xa4378818fe199cf14694deadcf64f72a55b11388e479f6e1fe65c1cd5122ed90</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785616850</t>
+          <t>1785622155</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>108.737864</t>
+          <t>3.30047</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd36df2627cc88fab7fdc1af73b8bcb3c0bf72929e79cf6bd4528a73bb336310c</t>
+          <t>0x7db9d72fe05e9c0b7cafae80909132292491f895d8118cd2683b7b765f885fc6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -862,12 +862,12 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>38.02995</t>
+          <t>23.76998</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.8588</t>
+          <t>1.7425</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -883,27 +883,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
+          <t>0xbef81e804b45a008094d3ed28e67d3330de2ca8be595e69a04b9ef716d1b1ec9</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -928,17 +928,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785616283</t>
+          <t>1785622131</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>44.28524</t>
+          <t>32.013441</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +955,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x5003aa71c29014639de94cd36c0d56636b10b1886f45c744d5d916eb60a6228c</t>
+          <t>0x39eb8621b888d9150a0d16c36b67e7d90727962020bed6edde941fa0cb4d01a1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -963,19 +963,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8.00529</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2338</t>
+          <t>1.5713</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -983,11 +979,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -995,27 +987,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
+          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1040,17 +1032,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785615140</t>
+          <t>1785618894</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>34.24723</t>
+          <t>8.595186</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1067,39 +1059,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x47ab07234e0925e967962637a863ed524a79d48b9d461f04f5d7dcb51a9077bd</t>
+          <t>0x1c5449fdfedcee8971c0c384741afccf1819625941cea175c42c57045be09079</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x1111084DE52322898FE58e14BCC4824Bf3fEbcfa</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8.01</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2325</t>
+          <t>1.1525</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1122,7 +1106,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
+          <t>0xc4044a0346c09a988a8646f1c19fcf4f0aebf02dd86358ff869417e13a149799</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1136,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785615140</t>
+          <t>1785617083</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1146,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>34.451613</t>
+          <t>11.344262</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,7 +1163,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x4a0fce837f4b39328cc4cb76d4060e94a4597f4078a1ad0dff75a038c5d092c3</t>
+          <t>0x49fe40db9721a6aaa44c12cdaa59de055cc21b9adc2a34ca866505256192b968</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1187,19 +1171,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>98</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.2338</t>
+          <t>1.875</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1207,11 +1187,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1234,7 +1210,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1264,7 +1240,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785615126</t>
+          <t>1785616859</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1274,7 +1250,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>4.278075</t>
+          <t>112.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,31 +1267,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xe7448cde3292b98680d8d685555b200090ccc908e6930965d17be8e6401d5629</t>
+          <t>0x4d5eee136de8446546eda81cbb34b3151a02e3a65539b580d186d7b15e7a047c</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.8325</t>
+          <t>1.1287</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Tecnico U.</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1323,27 +1307,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xb4df2c601601b81281545002a7ee9a847a424801fa9f9ea09b68e930c647c2b2</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1352,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785613773</t>
+          <t>1785616850</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.201201</t>
+          <t>108.737864</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,39 +1379,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xcac4d184a3b30b230068ae9c913c5c20aa85bbc70c10395795d8dd47887baf38</t>
+          <t>0xd36df2627cc88fab7fdc1af73b8bcb3c0bf72929e79cf6bd4528a73bb336310c</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>38.02995</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.5025</t>
+          <t>1.8588</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Universidad Catolica del Ecuador -1</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -1450,7 +1426,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0x31555f5a7bf5aa548ff66c4f2796f1137f0693f711b4b80344d2077fd6766592</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1480,7 +1456,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785608052</t>
+          <t>1785616283</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1466,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>19.900498</t>
+          <t>44.28524</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1483,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
+          <t>0x5003aa71c29014639de94cd36c0d56636b10b1886f45c744d5d916eb60a6228c</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1522,52 +1498,52 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.24999</t>
+          <t>8.00529</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1568,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785586109</t>
+          <t>1785615140</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2.48137</t>
+          <t>34.24723</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,12 +1595,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
+          <t>0x47ab07234e0925e967962637a863ed524a79d48b9d461f04f5d7dcb51a9077bd</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1634,52 +1610,52 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>115.96999</t>
+          <t>8.01</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.2325</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1680,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785581613</t>
+          <t>1785615140</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>233.692675</t>
+          <t>34.451613</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
+          <t>0x4a0fce837f4b39328cc4cb76d4060e94a4597f4078a1ad0dff75a038c5d092c3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1746,52 +1722,52 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>115.97</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.4963</t>
+          <t>1.2338</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Manta FC 0</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
+          <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1816,17 +1792,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785579320</t>
+          <t>1785615126</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>233.692695</t>
+          <t>4.278075</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1843,28 +1819,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
+          <t>0xe7448cde3292b98680d8d685555b200090ccc908e6930965d17be8e6401d5629</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16.07</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.8325</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Under/Over (5)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1875,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xb4df2c601601b81281545002a7ee9a847a424801fa9f9ea09b68e930c647c2b2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785559247</t>
+          <t>1785613773</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>29.554023</t>
+          <t>1.201201</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,23 +1923,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
+          <t>0xcac4d184a3b30b230068ae9c913c5c20aa85bbc70c10395795d8dd47887baf38</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0xf4a8B27C9a13e298D65b5Cc072d252816B799C81</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>16.07</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.5025</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1971,7 +1951,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Universidad Catolica del Ecuador -1</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2024,7 +2008,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785559247</t>
+          <t>1785608052</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2034,7 +2018,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>29.554023</t>
+          <t>19.900498</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,23 +2035,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
+          <t>0xd0a1fa503ade1da26d628202443f8fbf442918a501c47262abc2f7e2c7aedf1c</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.24999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5238</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2075,7 +2063,11 @@
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2098,7 +2090,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2128,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785559217</t>
+          <t>1785586109</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2138,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.909308</t>
+          <t>2.48137</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2155,7 +2147,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
+          <t>0x29e965d551245d9018463e50f9075f83b10aff02f39db068d1c37a5ff4723160</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2163,23 +2155,31 @@
           <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>15.99</t>
+          <t>115.96999</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2187,27 +2187,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2232,17 +2232,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785559203</t>
+          <t>1785581613</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>29.474654</t>
+          <t>233.692675</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2259,31 +2259,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
+          <t>0x36bdf43768d097bea2b6b7cf8c8eb40a364f6be26bcc2bdbc34a4358bd15f24a</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x358078dD5Ee4d532029b3cD743Bba2B6EFF8c6CA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>15.99</t>
+          <t>115.97</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.4963</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Manta FC 0</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -2291,27 +2299,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe3889fc065cfbda24effd8d65ae7dcf33bf6217b69edbfc67fe5a5410d79353b</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2336,17 +2344,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785559203</t>
+          <t>1785579320</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>29.474654</t>
+          <t>233.692695</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2363,7 +2371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
+          <t>0xb2e4c02e28211933f6b928f86cac2342a44028e4a06834899e2493f826b3d18d</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2374,12 +2382,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>15.83</t>
+          <t>16.07</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2440,7 +2448,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785559136</t>
+          <t>1785559247</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2450,7 +2458,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>29.314815</t>
+          <t>29.554023</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2467,7 +2475,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
+          <t>0x8684b80e20e5839ef45c647ced9fdb6ad817bd8ed8ee9f052ed9fb1e53314f20</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2478,12 +2486,12 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>15.83</t>
+          <t>16.07</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2544,7 +2552,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785559135</t>
+          <t>1785559247</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2554,7 +2562,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>29.314815</t>
+          <t>29.554023</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2571,28 +2579,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
+          <t>0x3d067f145172c50e59ca0b4e380527c6465e9e7bced485ec545a5a801da4f192</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5238</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2603,27 +2611,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Universidad Catolica del Ecuador</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Tecnico U.</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19606829</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2648,17 +2656,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785559114</t>
+          <t>1785559217</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1785619800</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>1.909308</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2675,7 +2683,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
+          <t>0xe49aa1402b07e6a57788597efc22d36ee0bc2a44d12f4a67ccad485901181f5c</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2686,17 +2694,17 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>15.99</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2722,7 +2730,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2752,7 +2760,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785559114</t>
+          <t>1785559203</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2762,7 +2770,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.474654</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2779,7 +2787,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
+          <t>0x112a021845fe9bf95e367a0f700b597eb7a83a0ba4ffbe214ad8927ed4f5ca3b</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2790,12 +2798,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>15.99</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2856,7 +2864,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785559105</t>
+          <t>1785559203</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2866,7 +2874,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.474654</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2883,7 +2891,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
+          <t>0xcd930a180859d9aa8e9ec5063039c25a51d1b84f426ce098fab2b826be43c14e</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2894,12 +2902,12 @@
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>15.67</t>
+          <t>15.83</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2960,7 +2968,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785559105</t>
+          <t>1785559136</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2970,7 +2978,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>29.153488</t>
+          <t>29.314815</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2987,28 +2995,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
+          <t>0x55c713e486fd070fd153fe7b8a4740d30756c92c24199ced6ae9a4fb21d66032</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>173.57</t>
+          <t>15.83</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3034,7 +3042,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3064,7 +3072,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785557644</t>
+          <t>1785559135</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3074,7 +3082,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>322.92093</t>
+          <t>29.314815</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3091,18 +3099,18 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
+          <t>0xa1be8be545a12de4b1d2eb30fc36822fcea98c5b6477da0386665686d8546491</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>173.57</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3112,7 +3120,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -3138,7 +3146,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3168,7 +3176,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785557643</t>
+          <t>1785559114</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3178,7 +3186,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>322.92093</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3195,39 +3203,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
+          <t>0x689ddef40b716c0d441f47a869b282dbf7e1f244a3db28a2be41cb4824098592</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2.34</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.4062</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785540081</t>
+          <t>1785559114</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>5.76</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3307,39 +3307,31 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
+          <t>0xffe8d26c7257da8b1458a45b7ac21e2ee10747a7829189f377bdbdd795abc7f3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.3313</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Libertad FC</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -3347,27 +3339,27 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -3392,17 +3384,17 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785524760</t>
+          <t>1785559105</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>3.018868</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3419,28 +3411,28 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
+          <t>0x1979af5cdf97b6ea5b2ba5732ba661a3af4f1eb07d15243486541a2391455fb2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.67</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.5913</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -3451,27 +3443,27 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Emelec vs Aucas</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Emelec</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Aucas</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>L19607503</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -3496,17 +3488,17 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785513340</t>
+          <t>1785559105</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>1785628800</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1.691332</t>
+          <t>29.153488</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3523,28 +3515,28 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
+          <t>0xebf29524cca596e42a9c958e8921be8876eeae25d2e79f7280c89fecef315b1e</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>173.57</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.6825</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Asian Handicap (-1.5)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -3555,27 +3547,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
+          <t>0xe4329a308902f0dc55a206367f7da0dd7eca95268d2af0c7d48cb5f71117e8d8</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3600,17 +3592,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785513160</t>
+          <t>1785557644</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.465201</t>
+          <t>322.92093</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3627,7 +3619,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
+          <t>0x27a2ff7d9b798a83f7ef4730f744085ed74d62b54823ad85bbbf1ec8a89aea9f</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3638,17 +3630,17 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>18.41999</t>
+          <t>173.57</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5537</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>LigaPro</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -3659,27 +3651,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
+          <t>0x23ca4379e0a47d5d152839e779d31257e03c01698f52329f5164b3eb1619224a</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3704,17 +3696,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785497374</t>
+          <t>1785557643</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>33.26409</t>
+          <t>322.92093</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3731,7 +3723,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
+          <t>0x9879a7b6cfc4fa023c72052a5b9881737a2eec7ddd2bd1d9bfeb15797c9d8925</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3746,22 +3738,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>2.34</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.3738</t>
+          <t>1.4062</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3771,27 +3763,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Tecnico U.</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
+          <t>0x066dc3fa4a3c8700f5683a34451f545686c5314e17533d096bcb8664c8b07137</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19606829</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3816,17 +3808,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785497256</t>
+          <t>1785540081</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785619800</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>4.120401</t>
+          <t>5.76</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3843,12 +3835,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
+          <t>0x572942571527f4a285d724ce3da87dc60480f515ece4ccc38a99dfb2599b1fb7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3858,12 +3850,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15.65</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.3738</t>
+          <t>1.3313</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3873,32 +3865,32 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Libertad FC vs Orense Sporting Club</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
           <t>Orense Sporting Club</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Libertad FC</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Orense Sporting Club</t>
-        </is>
-      </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3928,7 +3920,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785497255</t>
+          <t>1785524760</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3938,7 +3930,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>41.87291</t>
+          <t>3.018868</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3955,67 +3947,59 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
+          <t>0x3378821d00d0f476caa79caf9d32e8a08b63b698067887429774c9e1ced599de</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.5038</t>
+          <t>1.5913</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Libertad FC 0</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Libertad FC vs Orense Sporting Club</t>
+          <t>Emelec vs Aucas</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Emelec</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Orense Sporting Club</t>
+          <t>Aucas</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
+          <t>0xfb32031071813c746101fb9b0b752f058f1224fcef739c0a06325a255b6fd53e</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19614758</t>
+          <t>L19607503</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4040,17 +4024,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785487800</t>
+          <t>1785513340</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1785542400</t>
+          <t>1785628800</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>7.543424</t>
+          <t>1.691332</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4067,28 +4051,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
+          <t>0x12a039076c870c861492e25d9c04b652c8b4d4361cbc2283125f6def10853274</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+          <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.6825</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -4099,27 +4083,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xb211cc5404a48394b77e502360583ec16cd625ee74c5e5885308d65ddc497907</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4144,17 +4128,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785460511</t>
+          <t>1785513160</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>27.210884</t>
+          <t>1.465201</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4171,28 +4155,28 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
+          <t>0xa5b3d68b2642f8317db5aa6234979468ffd316702aa575ccca861a5abb45dbfa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>18.41999</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.3675</t>
+          <t>1.5537</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>LigaPro</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -4203,27 +4187,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xc414d1851d332f14f9b904e5e2f8963b17d626ab4fedbfd1d860c5ca0d8a5c2e</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4248,17 +4232,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785460290</t>
+          <t>1785497374</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>26.122449</t>
+          <t>33.26409</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4275,23 +4259,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
+          <t>0xf869759eb33d130e04144d3df7eb2a15b9e83af58f09e56bef9af7da2e867274</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.44982</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.3738</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4299,7 +4287,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Orense Sporting Club</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -4307,27 +4299,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4352,17 +4344,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785459886</t>
+          <t>1785497256</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>0.6426</t>
+          <t>4.120401</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4379,23 +4371,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
+          <t>0x6bf9bf6d90ab05711b64e3258529a8073c4bb1056bff9906eee709566f785280</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>463.04</t>
+          <t>15.65</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.3738</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4403,7 +4399,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Orense Sporting Club</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -4411,27 +4411,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xd8a8103adc6de6609b86d3c49639d966c7a1b009d923b1c33f1687d853406004</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4456,17 +4456,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785459772</t>
+          <t>1785497255</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>712.369231</t>
+          <t>41.87291</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4483,31 +4483,39 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
+          <t>0x91afdb3056b97dc838512da3006edc8d40d795e1cbf61754dd27b42bffbd9db4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>9.84</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.4363</t>
+          <t>1.5038</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Libertad FC 0</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -4515,27 +4523,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Libertad FC vs Orense Sporting Club</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Orense Sporting Club</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0xf805a6b6914a32854187614782fd2287c1f192abfc5aeb543744efbea5dd36e2</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19614758</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4560,17 +4568,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785459616</t>
+          <t>1785487800</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785542400</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>22.555874</t>
+          <t>7.543424</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4587,23 +4595,23 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
+          <t>0xcdbab7f720ecc2609cc986e33ee19c14fa06efd04db5f8d0ad2191eac40b0fc7</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4664,7 +4672,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785459612</t>
+          <t>1785460511</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4674,7 +4682,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>45.977011</t>
+          <t>27.210884</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4691,23 +4699,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
+          <t>0x8eed2f9e278deaeb4e1628ba136974f1228d0035db9cb9a273c6e2e8572240ac</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
+          <t>0x3287C9BCD7D05d027E8398cCAfE385a232D16B2C</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0.6173</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.4087</t>
+          <t>1.3675</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4768,7 +4776,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785459609</t>
+          <t>1785460290</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4778,7 +4786,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.510214</t>
+          <t>26.122449</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4795,28 +4803,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
+          <t>0x5cef349f9cfb08f0092efea94b1e1eba2316aeb489bcac201bd39d8fcdf537c8</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>0.44982</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -4827,27 +4835,27 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4872,17 +4880,17 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785459608</t>
+          <t>1785459886</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>112.676056</t>
+          <t>0.6426</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4899,28 +4907,28 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
+          <t>0x4ec9bf0ae9b293566857be0aa3d45d789368888ea7711a80eb74a83b16d81f4e</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>463.04</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -4931,27 +4939,27 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+          <t>Manta FC vs Mushuc Runa</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Leones Del Norte</t>
+          <t>Manta FC</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Barcelona Sporting Club</t>
+          <t>Mushuc Runa</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>L19615984</t>
+          <t>L19605615</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -4976,17 +4984,17 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785459600</t>
+          <t>1785459772</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>1785712200</t>
+          <t>1785610800</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>281.690141</t>
+          <t>712.369231</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5003,23 +5011,23 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
+          <t>0xbd33d07c10885c67a924c31f597f4aa5269e749d7ebe942f21e7126f5b3963fb</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+          <t>0x90aaAb8CC5139A43b5B8A6386929790Aa027Ab30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>9.84</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.4363</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5080,7 +5088,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785459599</t>
+          <t>1785459616</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5090,7 +5098,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>45.070423</t>
+          <t>22.555874</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5107,12 +5115,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+          <t>0x822816cff19781f933159cdf709b5e367523844ca5b9fd352afa4ced63e4f188</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+          <t>0x0c68d398894468F84ECb4805726f19c37e2B3415</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -5123,7 +5131,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.435</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5184,7 +5192,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1785459589</t>
+          <t>1785459612</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -5194,7 +5202,7 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>56.338028</t>
+          <t>45.977011</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -5211,23 +5219,23 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+          <t>0x112b0eec53123207d54d485755814cb85c7a0e1221a71fe48e719c11999f226b</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+          <t>0xB892ABBd5A3E0A440c0F94149848F2C1DDf05C5B</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0.6173</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.4087</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5288,7 +5296,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1785459589</t>
+          <t>1785459609</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -5298,7 +5306,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>22.535211</t>
+          <t>1.510214</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -5315,23 +5323,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+          <t>0x6d2158602245d1bbacc34a6453b10a1fe16d7c6af14c30668a211849eeb8ba5b</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+          <t>0x9CbF4a8A9EC2a8BABcaC7819e205a7B128798fAa</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>133.14</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.3475</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5347,27 +5355,27 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -5392,17 +5400,17 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1785459478</t>
+          <t>1785459608</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>383.136691</t>
+          <t>112.676056</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -5419,67 +5427,59 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+          <t>0x31f03e88b769cce674016ee1a73349f277ff02ed997281a0fac5b88a4adc21b5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x104A90467B551Fee945180a93e5f0f385c538A75</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>250.01</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.4812</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>LigaPro</t>
-        </is>
-      </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -5504,17 +5504,17 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1785441463</t>
+          <t>1785459600</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>519.501299</t>
+          <t>281.690141</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -5531,39 +5531,31 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+          <t>0xeaf9f248dc1ebc5d9a1f2fdbcc82110f148761403b799b4f1d66fdcd0611ef42</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x3509E838511034368Ed1aA44b85Bc5b1af675684</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>141.16</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.3438</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Manta FC</t>
-        </is>
-      </c>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>LigaPro</t>
@@ -5571,27 +5563,27 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Manta FC vs Mushuc Runa</t>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Manta FC</t>
+          <t>Leones Del Norte</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Mushuc Runa</t>
+          <t>Barcelona Sporting Club</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>L19605615</t>
+          <t>L19615984</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -5616,17 +5608,17 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1785441440</t>
+          <t>1785459599</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>1785610800</t>
+          <t>1785712200</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>410.647273</t>
+          <t>45.070423</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -5643,110 +5635,646 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>0xe0216d65c84aa6a069cef40fe70d14810fef09d2e27e600aa1801d2b644c168e</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0xD19384284ACEe246037b2f52b50EEF17F1e33B74</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>56.338028</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0x5386cc079cbea6f8024fcb1f4fd8c125fdb9c4d4507d7d72667521bc2234711c</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0xefEd5719272d06dDD2e1e383C3076aa8262a2C55</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1.355</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Leones Del Norte vs Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Leones Del Norte</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Barcelona Sporting Club</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>0xaa6e0d011cd1f0f90445686073986da2b91bd350bd98d5463185fb2d4823b6c3</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>L19615984</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1785459589</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>1785712200</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>22.535211</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0x588486ac7bdc3d012f0c913f77b7dabec6ba1e59371770a8a166aede4963f976</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0x24B2465f0c768EdAA0DEBbb7DB5C6345239F7d87</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>133.14</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1.3475</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>0x28d74792b0065ec6861aca96e85c560a964fd866c6e9a22a3d23b26ddaaee489</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>1785459478</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>383.136691</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0x7309daf787ae3e353d988657b675fea72aff1d7086065c258d3c16a3a73012a8</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>250.01</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1.4812</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>0x8eedc564abb7307b4ef89fa66291601295b22578d5296ac8e0af172b47a57d7c</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>1785441463</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>519.501299</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0x1f7f2d61f5529a2354ab2c3ca0ce271c1931037e2901585e390e07f87e506ee0</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0xF974DAF59EA0cdfBD2125EcBB5BacEBA8F4727dA</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>141.16</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1.3438</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>LigaPro</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Manta FC vs Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Manta FC</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>0x6bb6296b7aec74167b3bd11b6c86d525a8bef7b59c2155a1e98611017de1a15f</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>L19605615</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>1785441440</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>1785610800</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>410.647273</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>0x6599044f3d4d50487489b07a035618092f1d03440ffd54856dcd903844650bb5</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>0x44a80DC6b2015FBaC7a505fB0D7CCa1FAC58C7Bf</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>1.2575</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>1X2</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>Tie</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>LigaPro</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador vs Tecnico U.</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>Universidad Catolica del Ecuador</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>Tecnico U.</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>0x6f48cb9ab2adc3f80f8a9cce4985a85384a62c4eb9ef39c2fcda8ffbe498fcac</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>L19606829</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr">
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
         <is>
           <t>1785344362</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="S55" t="inlineStr">
         <is>
           <t>1785619800</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="T55" t="inlineStr">
         <is>
           <t>3.883495</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="U55" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr">
+      <c r="V55" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>